<commit_message>
claude successfully fixed fem.py
</commit_message>
<xml_diff>
--- a/docs/inputs/slope/xslope_dam.xlsx
+++ b/docs/inputs/slope/xslope_dam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD9A34F6-2305-8148-9B25-886396FD56A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97918473-CDAC-8249-B887-D140C850231F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27920" yWindow="2240" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="27920" yWindow="2240" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -937,7 +937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1085,6 +1085,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9626,8 +9629,12 @@
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
+      <c r="W9" s="54">
+        <v>700000</v>
+      </c>
+      <c r="X9" s="3">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
@@ -9670,8 +9677,12 @@
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
+      <c r="W10" s="54">
+        <v>700000</v>
+      </c>
+      <c r="X10" s="3">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
@@ -9714,8 +9725,12 @@
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
-      <c r="X11" s="3"/>
+      <c r="W11" s="54">
+        <v>700000</v>
+      </c>
+      <c r="X11" s="3">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="3">

</xml_diff>

<commit_message>
updated earth dam files to proper max depth
</commit_message>
<xml_diff>
--- a/docs/inputs/slope/xslope_dam.xlsx
+++ b/docs/inputs/slope/xslope_dam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97918473-CDAC-8249-B887-D140C850231F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5C36CB-4225-7D49-BBC5-C3F95D601ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27920" yWindow="2240" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="27920" yWindow="2240" windowWidth="34200" windowHeight="20240" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="157">
   <si>
     <t>X</t>
   </si>
@@ -390,9 +390,6 @@
     <t>d</t>
   </si>
   <si>
-    <t>ψ</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -411,9 +408,6 @@
       </rPr>
       <t>(d)</t>
     </r>
-  </si>
-  <si>
-    <t>s(ψ)</t>
   </si>
   <si>
     <t>Piezometric Line 2</t>
@@ -670,7 +664,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -788,6 +782,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="16">
@@ -1084,19 +1083,22 @@
     <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1116,9 +1118,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8093,7 +8092,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
@@ -8110,11 +8109,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -8130,10 +8129,10 @@
         <v>62.4</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -8205,10 +8204,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F15" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G15" t="s">
         <v>123</v>
-      </c>
-      <c r="G15" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -8222,18 +8221,18 @@
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
       <c r="F17" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G18" s="9" t="s">
         <v>124</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
@@ -8267,34 +8266,34 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="F2" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="32" t="s">
+        <v>111</v>
+      </c>
+      <c r="I2" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2" s="33" t="s">
+        <v>101</v>
+      </c>
+      <c r="K2" s="33" t="s">
         <v>107</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="F2" s="32" t="s">
-        <v>110</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="H2" s="32" t="s">
-        <v>113</v>
-      </c>
-      <c r="I2" s="32" t="s">
-        <v>114</v>
-      </c>
-      <c r="J2" s="33" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="33" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -8553,7 +8552,7 @@
       <c r="K19" s="3"/>
       <c r="M19" s="31"/>
       <c r="N19" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
@@ -8572,7 +8571,7 @@
       <c r="K20" s="3"/>
       <c r="M20" s="34"/>
       <c r="N20" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
@@ -8633,54 +8632,54 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="52" t="s">
-        <v>140</v>
-      </c>
-      <c r="C2" s="52"/>
-      <c r="E2" s="48" t="s">
+      <c r="B2" s="53" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" s="53"/>
+      <c r="E2" s="49" t="s">
+        <v>133</v>
+      </c>
+      <c r="F2" s="49"/>
+      <c r="H2" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="I2" s="49"/>
+      <c r="K2" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="F2" s="48"/>
-      <c r="H2" s="48" t="s">
+      <c r="L2" s="49"/>
+      <c r="N2" s="49" t="s">
         <v>136</v>
       </c>
-      <c r="I2" s="48"/>
-      <c r="K2" s="48" t="s">
+      <c r="O2" s="49"/>
+      <c r="Q2" s="49" t="s">
         <v>137</v>
       </c>
-      <c r="L2" s="48"/>
-      <c r="N2" s="48" t="s">
-        <v>138</v>
-      </c>
-      <c r="O2" s="48"/>
-      <c r="Q2" s="48" t="s">
-        <v>139</v>
-      </c>
-      <c r="R2" s="48"/>
+      <c r="R2" s="49"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
+      <c r="B3" s="53"/>
+      <c r="C3" s="53"/>
       <c r="E3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F3" s="38">
         <v>302</v>
       </c>
       <c r="H3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I3" s="38"/>
       <c r="K3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L3" s="38"/>
       <c r="N3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="O3" s="38"/>
       <c r="Q3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="R3" s="38"/>
     </row>
@@ -9053,52 +9052,52 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="54" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="54"/>
+      <c r="E2" s="50" t="s">
+        <v>139</v>
+      </c>
+      <c r="F2" s="50"/>
+      <c r="H2" s="50" t="s">
+        <v>141</v>
+      </c>
+      <c r="I2" s="50"/>
+      <c r="K2" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="E2" s="49" t="s">
-        <v>141</v>
-      </c>
-      <c r="F2" s="49"/>
-      <c r="H2" s="49" t="s">
+      <c r="L2" s="50"/>
+      <c r="N2" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="I2" s="49"/>
-      <c r="K2" s="49" t="s">
+      <c r="O2" s="50"/>
+      <c r="Q2" s="50" t="s">
         <v>144</v>
       </c>
-      <c r="L2" s="49"/>
-      <c r="N2" s="49" t="s">
-        <v>145</v>
-      </c>
-      <c r="O2" s="49"/>
-      <c r="Q2" s="49" t="s">
-        <v>146</v>
-      </c>
-      <c r="R2" s="49"/>
+      <c r="R2" s="50"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
       <c r="E3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F3" s="40"/>
       <c r="H3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I3" s="40"/>
       <c r="K3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L3" s="40"/>
       <c r="N3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="O3" s="40"/>
       <c r="Q3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="R3" s="40"/>
     </row>
@@ -9464,7 +9463,7 @@
       <c r="E2"/>
       <c r="F2"/>
       <c r="J2" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="O2" s="6"/>
     </row>
@@ -9478,7 +9477,7 @@
       <c r="E3"/>
       <c r="F3"/>
       <c r="J3" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="K3" t="s">
         <v>59</v>
@@ -9504,10 +9503,10 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="J5" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="O5" s="14"/>
     </row>
@@ -9538,14 +9537,14 @@
       <c r="P7" s="44"/>
       <c r="Q7" s="44"/>
       <c r="R7" s="44" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="S7" s="44"/>
       <c r="T7" s="44"/>
       <c r="U7" s="44"/>
       <c r="V7" s="44"/>
       <c r="W7" s="44" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="X7" s="44"/>
     </row>
@@ -9578,10 +9577,10 @@
         <v>80</v>
       </c>
       <c r="J8" s="21" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="K8" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="L8" s="22" t="s">
         <v>54</v>
@@ -9596,31 +9595,31 @@
         <v>74</v>
       </c>
       <c r="P8" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Q8" s="23" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="R8" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="S8" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="T8" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="S8" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="T8" s="25" t="s">
-        <v>94</v>
-      </c>
       <c r="U8" s="25" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="V8" s="25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="W8" s="29" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="X8" s="30" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
@@ -9628,7 +9627,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C9" s="3">
         <v>125</v>
@@ -9660,7 +9659,7 @@
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
-      <c r="W9" s="54">
+      <c r="W9" s="43">
         <v>700000</v>
       </c>
       <c r="X9" s="3">
@@ -9672,7 +9671,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C10" s="3">
         <v>122</v>
@@ -9708,7 +9707,7 @@
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
-      <c r="W10" s="54">
+      <c r="W10" s="43">
         <v>700000</v>
       </c>
       <c r="X10" s="3">
@@ -9720,7 +9719,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C11" s="3">
         <v>123</v>
@@ -9756,7 +9755,7 @@
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
-      <c r="W11" s="54">
+      <c r="W11" s="43">
         <v>700000</v>
       </c>
       <c r="X11" s="3">
@@ -9768,7 +9767,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C12" s="3">
         <v>127</v>
@@ -10472,266 +10471,266 @@
         <v>46</v>
       </c>
       <c r="B2" s="3">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="D4" s="47" t="s">
+      <c r="B4" s="46"/>
+      <c r="D4" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="47"/>
-      <c r="G4" s="47" t="s">
+      <c r="E4" s="46"/>
+      <c r="G4" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="47"/>
-      <c r="J4" s="47" t="s">
+      <c r="H4" s="46"/>
+      <c r="J4" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="47"/>
-      <c r="M4" s="47" t="s">
+      <c r="K4" s="46"/>
+      <c r="M4" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="47"/>
-      <c r="P4" s="47" t="s">
+      <c r="N4" s="46"/>
+      <c r="P4" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="47"/>
+      <c r="Q4" s="46"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="47" t="s">
+      <c r="S4" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="47"/>
+      <c r="T4" s="46"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="47" t="s">
+      <c r="V4" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="47"/>
+      <c r="W4" s="46"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="47" t="s">
+      <c r="Y4" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="47"/>
+      <c r="Z4" s="46"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="47" t="s">
+      <c r="AB4" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="47"/>
-      <c r="AE4" s="47" t="s">
+      <c r="AC4" s="46"/>
+      <c r="AE4" s="46" t="s">
+        <v>114</v>
+      </c>
+      <c r="AF4" s="46"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="46" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI4" s="46"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="46" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="47"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="47" t="s">
+      <c r="AL4" s="46"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="AI4" s="47"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="47" t="s">
+      <c r="AO4" s="46"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="46" t="s">
         <v>118</v>
       </c>
-      <c r="AL4" s="47"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="47" t="s">
-        <v>119</v>
-      </c>
-      <c r="AO4" s="47"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="AR4" s="47"/>
+      <c r="AR4" s="46"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B5" s="42">
         <v>1</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E5" s="42">
         <v>2</v>
       </c>
       <c r="G5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H5" s="42">
         <v>3</v>
       </c>
       <c r="J5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K5" s="42">
         <v>4</v>
       </c>
       <c r="M5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="N5" s="42">
         <v>5</v>
       </c>
       <c r="P5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Q5" s="42">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="T5" s="42">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="W5" s="42">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Z5" s="42">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AC5" s="42">
         <v>10</v>
       </c>
       <c r="AE5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AF5" s="42">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AI5" s="42">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AL5" s="42">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AO5" s="42">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AR5" s="42">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="45" t="str">
+      <c r="A6" s="47" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Shell</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="D6" s="45" t="str">
+      <c r="B6" s="48"/>
+      <c r="D6" s="47" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Core</v>
       </c>
-      <c r="E6" s="46"/>
-      <c r="G6" s="45" t="str">
+      <c r="E6" s="48"/>
+      <c r="G6" s="47" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Clay</v>
       </c>
-      <c r="H6" s="46"/>
-      <c r="J6" s="45" t="str">
+      <c r="H6" s="48"/>
+      <c r="J6" s="47" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>Sand</v>
       </c>
-      <c r="K6" s="46"/>
-      <c r="M6" s="45" t="str">
+      <c r="K6" s="48"/>
+      <c r="M6" s="47" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="46"/>
-      <c r="P6" s="45" t="str">
+      <c r="N6" s="48"/>
+      <c r="P6" s="47" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="46"/>
+      <c r="Q6" s="48"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="45" t="str">
+      <c r="S6" s="47" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="46"/>
+      <c r="T6" s="48"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="45" t="str">
+      <c r="V6" s="47" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="46"/>
+      <c r="W6" s="48"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="45" t="str">
+      <c r="Y6" s="47" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="46"/>
+      <c r="Z6" s="48"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="45" t="str">
+      <c r="AB6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="46"/>
-      <c r="AE6" s="45" t="str">
+      <c r="AC6" s="48"/>
+      <c r="AE6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="46"/>
+      <c r="AF6" s="48"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="45" t="str">
+      <c r="AH6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="46"/>
+      <c r="AI6" s="48"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="45" t="str">
+      <c r="AK6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="46"/>
+      <c r="AL6" s="48"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="45" t="str">
+      <c r="AN6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="46"/>
+      <c r="AO6" s="48"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="45" t="str">
+      <c r="AQ6" s="47" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="46"/>
+      <c r="AR6" s="48"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11683,36 +11682,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11728,16 +11727,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="48" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" s="48"/>
-      <c r="D2" s="49" t="s">
+      <c r="A2" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="49"/>
+      <c r="B2" s="49"/>
+      <c r="D2" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="50"/>
       <c r="G2" s="24" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -12314,36 +12313,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="51" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="F2" s="51" t="s">
+        <v>128</v>
+      </c>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="J2" s="51" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="F2" s="50" t="s">
+      <c r="K2" s="51"/>
+      <c r="L2" s="51"/>
+      <c r="N2" s="51" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="J2" s="50" t="s">
+      <c r="O2" s="51"/>
+      <c r="P2" s="51"/>
+      <c r="R2" s="51" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
-      <c r="N2" s="50" t="s">
+      <c r="S2" s="51"/>
+      <c r="T2" s="51"/>
+      <c r="V2" s="51" t="s">
         <v>132</v>
       </c>
-      <c r="O2" s="50"/>
-      <c r="P2" s="50"/>
-      <c r="R2" s="50" t="s">
-        <v>133</v>
-      </c>
-      <c r="S2" s="50"/>
-      <c r="T2" s="50"/>
-      <c r="V2" s="50" t="s">
-        <v>134</v>
-      </c>
-      <c r="W2" s="50"/>
-      <c r="X2" s="50"/>
+      <c r="W2" s="51"/>
+      <c r="X2" s="51"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -12832,36 +12831,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="52" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="F2" s="52" t="s">
+        <v>146</v>
+      </c>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="J2" s="52" t="s">
         <v>147</v>
       </c>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="F2" s="51" t="s">
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="N2" s="52" t="s">
         <v>148</v>
       </c>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="J2" s="51" t="s">
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+      <c r="R2" s="52" t="s">
         <v>149</v>
       </c>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
-      <c r="N2" s="51" t="s">
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="V2" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="P2" s="51"/>
-      <c r="R2" s="51" t="s">
-        <v>151</v>
-      </c>
-      <c r="S2" s="51"/>
-      <c r="T2" s="51"/>
-      <c r="V2" s="51" t="s">
-        <v>152</v>
-      </c>
-      <c r="W2" s="51"/>
-      <c r="X2" s="51"/>
+      <c r="W2" s="52"/>
+      <c r="X2" s="52"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>